<commit_message>
Neutral sample cities/emails/phones; regenerate GIF without unsourced time-saved figure
</commit_message>
<xml_diff>
--- a/cleanup_demo.xlsx
+++ b/cleanup_demo.xlsx
@@ -653,7 +653,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>springfield</t>
+          <t>boston</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Boston</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>SPRINGFIELD</t>
+          <t>BOSTON</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,6 @@
           <t>Carol Nguyen</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>555.0103</t>
@@ -760,7 +759,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>lyon</t>
+          <t>denver</t>
         </is>
       </c>
     </row>
@@ -797,7 +796,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>marseille</t>
+          <t>seattle</t>
         </is>
       </c>
     </row>
@@ -832,7 +831,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -867,7 +865,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>springfield</t>
+          <t>boston</t>
         </is>
       </c>
     </row>
@@ -879,12 +877,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>f.zahra@mail.fr</t>
+          <t>f.zahra@mail.io</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>06 12 34 56 78</t>
+          <t>+44 7700 900123</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -904,12 +902,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Austin</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>ghost@x.com</t>
@@ -937,7 +934,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Miami</t>
         </is>
       </c>
     </row>
@@ -949,7 +946,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>hugo@blanc.fr</t>
+          <t>hugo@blanc.io</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -974,7 +971,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>bordeaux</t>
+          <t>chicago</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1079,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1122,7 +1119,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1137,7 +1134,6 @@
           <t>Carol Nguyen</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>5550103</t>
@@ -1158,7 +1154,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1198,10 +1194,9 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Marseille</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>Seattle</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1233,12 +1228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>f.zahra@mail.fr</t>
+          <t>f.zahra@mail.io</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0612345678</t>
+          <t>447700900123</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1256,12 +1251,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>FR decimal comma fixed</t>
+          <t>European decimal comma fixed</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1268,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hugo@blanc.fr</t>
+          <t>hugo@blanc.io</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1296,10 +1291,9 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>Chicago</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1329,6 +1323,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1411,6 +1406,8 @@
         <v>1400.75</v>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -1453,6 +1450,8 @@
         <v>1</v>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -1502,10 +1501,11 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Mode d'emploi / How to use</t>
-        </is>
-      </c>
-    </row>
+          <t>How to use</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>